<commit_message>
feat: Enhance schedule management with company trades and status filtering
- Added functionality to attach company trades to schedules in export and admin dashboard.
- Introduced status filtering for schedules in API endpoints and admin dashboard.
- Updated types to include primary trades and modified related components.
- Enhanced Excel export to include a new "職種" (trade) column.
- Improved user interface for selecting primary and secondary companies with datalist support.
- Added a new template for company master CSV to include trades.
</commit_message>
<xml_diff>
--- a/ktnk/excel/作業予定マスタ.xlsx
+++ b/ktnk/excel/作業予定マスタ.xlsx
@@ -86,12 +86,13 @@
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="8" width="20" customWidth="1"/>
-    <col min="9" max="14" width="18" customWidth="1"/>
-    <col min="15" max="18" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="9" width="20" customWidth="1"/>
+    <col min="10" max="15" width="18" customWidth="1"/>
+    <col min="16" max="19" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -117,6 +118,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -141,6 +143,7 @@
       <c r="P2"/>
       <c r="Q2"/>
       <c r="R2"/>
+      <c r="S2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -169,6 +172,7 @@
       <c r="P3"/>
       <c r="Q3"/>
       <c r="R3"/>
+      <c r="S3"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -197,6 +201,7 @@
       <c r="P4"/>
       <c r="Q4"/>
       <c r="R4"/>
+      <c r="S4"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -225,6 +230,7 @@
       <c r="P5"/>
       <c r="Q5"/>
       <c r="R5"/>
+      <c r="S5"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -253,6 +259,7 @@
       <c r="P6"/>
       <c r="Q6"/>
       <c r="R6"/>
+      <c r="S6"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -281,6 +288,7 @@
       <c r="P7"/>
       <c r="Q7"/>
       <c r="R7"/>
+      <c r="S7"/>
     </row>
     <row r="8">
       <c r="A8"/>
@@ -301,6 +309,7 @@
       <c r="P8"/>
       <c r="Q8"/>
       <c r="R8"/>
+      <c r="S8"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -329,9 +338,10 @@
       <c r="P9"/>
       <c r="Q9"/>
       <c r="R9"/>
+      <c r="S9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1"/>
+  <autoFilter ref="A1:S1"/>
 </worksheet>
 </file>
 
@@ -341,12 +351,13 @@
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="8" width="20" customWidth="1"/>
-    <col min="9" max="14" width="18" customWidth="1"/>
-    <col min="15" max="18" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="9" width="20" customWidth="1"/>
+    <col min="10" max="15" width="18" customWidth="1"/>
+    <col min="16" max="19" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -367,82 +378,87 @@
       </c>
       <c r="D1" t="inlineStr" s="2">
         <is>
+          <t>職種</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="2">
+        <is>
           <t>一次会社人数</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="2">
+      <c r="F1" t="inlineStr" s="2">
         <is>
           <t>二次会社</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="2">
+      <c r="G1" t="inlineStr" s="2">
         <is>
           <t>二次会社人数</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="2">
+      <c r="H1" t="inlineStr" s="2">
         <is>
           <t>作業エリア</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="2">
+      <c r="I1" t="inlineStr" s="2">
         <is>
           <t>作業内容</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="2">
+      <c r="J1" t="inlineStr" s="2">
         <is>
           <t>来場予定日</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="2">
+      <c r="K1" t="inlineStr" s="2">
         <is>
           <t>来場予定一次会社人数</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="2">
+      <c r="L1" t="inlineStr" s="2">
         <is>
           <t>来場予定二次会社</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="2">
+      <c r="M1" t="inlineStr" s="2">
         <is>
           <t>来場予定二次会社人数</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="2">
+      <c r="N1" t="inlineStr" s="2">
         <is>
           <t>来場予定作業エリア</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr" s="2">
+      <c r="O1" t="inlineStr" s="2">
         <is>
           <t>来場予定作業内容</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr" s="2">
+      <c r="P1" t="inlineStr" s="2">
         <is>
           <t>登録日時</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="2">
+      <c r="Q1" t="inlineStr" s="2">
         <is>
           <t>更新日時</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="2">
+      <c r="R1" t="inlineStr" s="2">
         <is>
           <t>取込日時</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="2">
+      <c r="S1" t="inlineStr" s="2">
         <is>
           <t>取込元ファイル</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1"/>
+  <autoFilter ref="A1:S1"/>
 </worksheet>
 </file>
 
@@ -452,12 +468,13 @@
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="8" width="20" customWidth="1"/>
-    <col min="9" max="14" width="18" customWidth="1"/>
-    <col min="15" max="18" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="9" width="20" customWidth="1"/>
+    <col min="10" max="15" width="18" customWidth="1"/>
+    <col min="16" max="19" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,75 +495,80 @@
       </c>
       <c r="D1" t="inlineStr" s="2">
         <is>
+          <t>職種</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="2">
+        <is>
           <t>一次会社人数</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="2">
+      <c r="F1" t="inlineStr" s="2">
         <is>
           <t>二次会社</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr" s="2">
+      <c r="G1" t="inlineStr" s="2">
         <is>
           <t>二次会社人数</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr" s="2">
+      <c r="H1" t="inlineStr" s="2">
         <is>
           <t>作業エリア</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr" s="2">
+      <c r="I1" t="inlineStr" s="2">
         <is>
           <t>作業内容</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr" s="2">
+      <c r="J1" t="inlineStr" s="2">
         <is>
           <t>来場予定日</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr" s="2">
+      <c r="K1" t="inlineStr" s="2">
         <is>
           <t>来場予定一次会社人数</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr" s="2">
+      <c r="L1" t="inlineStr" s="2">
         <is>
           <t>来場予定二次会社</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr" s="2">
+      <c r="M1" t="inlineStr" s="2">
         <is>
           <t>来場予定二次会社人数</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr" s="2">
+      <c r="N1" t="inlineStr" s="2">
         <is>
           <t>来場予定作業エリア</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr" s="2">
+      <c r="O1" t="inlineStr" s="2">
         <is>
           <t>来場予定作業内容</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr" s="2">
+      <c r="P1" t="inlineStr" s="2">
         <is>
           <t>登録日時</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr" s="2">
+      <c r="Q1" t="inlineStr" s="2">
         <is>
           <t>更新日時</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr" s="2">
+      <c r="R1" t="inlineStr" s="2">
         <is>
           <t>取込日時</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr" s="2">
+      <c r="S1" t="inlineStr" s="2">
         <is>
           <t>取込元ファイル</t>
         </is>
@@ -570,47 +592,52 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>配管工</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>△△工業</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>10F</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>配管施工</t>
         </is>
       </c>
-      <c r="I2"/>
       <c r="J2"/>
       <c r="K2"/>
       <c r="L2"/>
       <c r="M2"/>
       <c r="N2"/>
-      <c r="O2" t="inlineStr">
+      <c r="O2"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>2026-09-03 18:00</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>2026-09-03 18:00</t>
         </is>
       </c>
-      <c r="Q2"/>
       <c r="R2"/>
+      <c r="S2"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -630,47 +657,52 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>配管工</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>□□工業</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>10F</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>配管施工</t>
         </is>
       </c>
-      <c r="I3"/>
       <c r="J3"/>
       <c r="K3"/>
       <c r="L3"/>
       <c r="M3"/>
       <c r="N3"/>
-      <c r="O3" t="inlineStr">
+      <c r="O3"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>2026-09-03 18:00</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>2026-09-03 18:00</t>
         </is>
       </c>
-      <c r="Q3"/>
       <c r="R3"/>
+      <c r="S3"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -688,55 +720,60 @@
           <t>○○設備</t>
         </is>
       </c>
-      <c r="D4"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>配管工</t>
+        </is>
+      </c>
       <c r="E4"/>
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4"/>
-      <c r="I4" t="inlineStr">
+      <c r="I4"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>△△工業</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>11F</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>配管施工</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>2026-09-03 18:00</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>2026-09-03 18:00</t>
         </is>
       </c>
-      <c r="Q4"/>
       <c r="R4"/>
+      <c r="S4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R1"/>
+  <autoFilter ref="A1:S1"/>
 </worksheet>
 </file>
</xml_diff>